<commit_message>
fix: match col names to bw node fields
</commit_message>
<xml_diff>
--- a/data/input-data-template.xlsx
+++ b/data/input-data-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yohan LANIER\Documents\Github\reduced-lci-extractor\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7CF44C-0B43-4889-8642-9E233BF20BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEAC4F21-2667-4977-B502-1B9AB51D09D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="activities" sheetId="1" r:id="rId1"/>
@@ -31,19 +31,19 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>activity name</t>
-  </si>
-  <si>
     <t>location</t>
-  </si>
-  <si>
-    <t>reference_product</t>
   </si>
   <si>
     <t>method_name</t>
   </si>
   <si>
     <t>impact_cat_name</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>reference product</t>
   </si>
 </sst>
 </file>
@@ -371,13 +371,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -396,10 +396,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>